<commit_message>
fix: customer profile edit modal save & direct client H: drive file mirror sync with lock fallback
</commit_message>
<xml_diff>
--- a/data/aba/Customer_Bank_Account_Number.xlsx
+++ b/data/aba/Customer_Bank_Account_Number.xlsx
@@ -32,8 +32,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0;#,##0"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -459,7 +460,7 @@
         <v/>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>087 777 345</v>
       </c>
       <c r="H2" t="str">
         <v>ផ្សាបឺងបៃតង</v>
@@ -4027,7 +4028,7 @@
         <v/>
       </c>
       <c r="G125" t="str">
-        <v/>
+        <v>Dr. Chea Chen Tong</v>
       </c>
       <c r="H125" t="str">
         <v>Takeo, Near Chouk</v>
@@ -9972,7 +9973,7 @@
         <v/>
       </c>
       <c r="G330" t="str">
-        <v/>
+        <v>Dr. Hab Mi</v>
       </c>
       <c r="H330" t="str">
         <v># KIRIRUM</v>
@@ -10784,7 +10785,7 @@
         <v/>
       </c>
       <c r="G358" t="str">
-        <v/>
+        <v>Dr. HENG MENG</v>
       </c>
       <c r="H358" t="str">
         <v>ST. 371, PC Market</v>
@@ -12582,7 +12583,7 @@
         <v/>
       </c>
       <c r="G420" t="str">
-        <v/>
+        <v>Dr. Houy Kheang</v>
       </c>
       <c r="H420" t="str">
         <v>Takmao</v>
@@ -15279,7 +15280,7 @@
         <v/>
       </c>
       <c r="G513" t="str">
-        <v/>
+        <v>Dr. Kim Hak</v>
       </c>
       <c r="H513" t="str">
         <v>ផ្ទះលេខ 84​ ផ្លូវ268 សង្កាត់ទឹកល្អក់3 ខណ្ឌទួលគោក រាជធានីភ្នំពេញ (សំណង់12)</v>
@@ -23979,7 +23980,7 @@
         <v/>
       </c>
       <c r="G813" t="str">
-        <v/>
+        <v>077 267 868</v>
       </c>
       <c r="H813" t="str">
         <v>#101, S.Phnom Penh Thmei, K.Sen Sok Phnom Penh Cambodia 12101</v>
@@ -34129,7 +34130,7 @@
         <v/>
       </c>
       <c r="G1163" t="str">
-        <v/>
+        <v>017 593 849</v>
       </c>
       <c r="H1163" t="str">
         <v>Siem Reap</v>
@@ -37232,7 +37233,7 @@
         <v/>
       </c>
       <c r="G1270" t="str">
-        <v/>
+        <v>Dr. Tem Chhou Heng</v>
       </c>
       <c r="H1270" t="str">
         <v>#95A, S.Phnom Penh Thmei, K.Sen Sok Phnom Penh Cambodia 12101</v>
@@ -46688,7 +46689,7 @@
         <v/>
       </c>
       <c r="G1596" t="str">
-        <v/>
+        <v>Dr. Ouk Davin</v>
       </c>
       <c r="H1596" t="str">
         <v>University of Health Sciences</v>
@@ -61598,7 +61599,7 @@
         <v/>
       </c>
       <c r="G2110" t="str">
-        <v/>
+        <v>Test</v>
       </c>
       <c r="H2110" t="str">
         <v/>

</xml_diff>